<commit_message>
INT-22: add ODM contract mapping (4 sheets) + ODM SOQL queries
Add ODM README, ODM Canonical Mapping (CREATE_SO), ODM File Mapping
(ODM_SS_STIFS RCTI extract) and ODM SOQL Queries sheets to the mapping
workbook; extend the SOQL markdown with the ODM CREATE_SO and RCTI
pull queries.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NUogd2hZimCwR1pqCdqWGg
</commit_message>
<xml_diff>
--- a/INT-22_Contract_Reference_Mapping_20260805.xlsx
+++ b/INT-22_Contract_Reference_Mapping_20260805.xlsx
@@ -13,6 +13,10 @@
     <sheet name="NBN Field Mapping" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Optus Field Mapping" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SOQL Queries" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ODM README" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ODM Canonical Mapping" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ODM File Mapping" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ODM SOQL Queries" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -676,6 +680,171 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>SOQL (SAP CPI Salesforce adapter)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Field -&gt; Target</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Notes / To confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="300" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>CREATE_SO</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>ODM Service Order / WBS creation — pull new ODM projects</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       Project_Name__c,
+       Address__c,
+       Description__c,
+       Project_Start_A__c,
+       sitetracker__Project_Status__c,
+       Business_Flow_Type__c,
+       Work_Type__c,
+       Job_Type__c,
+       State__c,
+       Region__c,
+       CCR__c,
+       CreatedDate, LastModifiedDate
+FROM sitetracker__Project__c
+WHERE CreatedDate &gt;= ${lastSuccessfulPullTimestamp}</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Constant 'CREATE_SO' -&gt; header.sourceMessageType
+Project_Name__c -&gt; header.fsmJobNumber / header.clientJobNumber
+CCR__c -&gt; header.clientContractId
+Work_Type__c (or cost code) -&gt; header.serviceHierarchy
+Job_Type__c -&gt; item.serviceHierarchy2
+State__c -&gt; header.state
+Region__c -&gt; header.customerRegion</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Base project pull validated in POC (connectivity + delta query on sitetracker__Project__c).
+CCR__c does NOT exist yet — field to be created in SiteTracker (GAP).
+Work_Type__c / Job_Type__c / State__c / Region__c API names proposed from labels — confirm with Jackie; verify whether serviceHierarchy source is workType or costCode.
+Optionally filter on status (Active/Released) per requirements matrix row 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="300" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>RCTI</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Supplier invoice — pull invoiced jobs + lines (replaces ODM_SS_STIFS file)</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       sitetracker__Job__c,
+       sitetracker__Job__r.Name,
+       sitetracker__Job__r.Project_Name__c,
+       sitetracker__Job__r.Date_Job_Invoiced__c,
+       sitetracker__Job__r.Total_Job_Amount__c,
+       sitetracker__Job__r.Business_Flow_Type__c,
+       sitetracker__Job__r.sitetracker__Vendor__r.Vendor_ID__c,
+       sitetracker__Job__r.sitetracker__Vendor__r.Name,
+       sitetracker__Job__r.Project__r.Project_Name__c,
+       sitetracker__Job__r.Project__r.Address__c,
+       Item_Name__r.Item_Id__c,
+       Item_Name__r.sitetracker__Primary_UoM__c,
+       Subie_Rate__c,
+       Total_Actual_Amount__c,
+       LastModifiedDate
+FROM sitetracker__Production_Plan_Line__c
+WHERE sitetracker__Job__r.sitetracker__Job_Status__c = 'Invoiced'
+  AND (LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp}
+       OR sitetracker__Job__r.LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp})</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Vendor_ID__c -&gt; supplier (file col 2, account.vendor_id__c)
+Job Name -&gt; invoice line key (file cols 3/4/24, job.name)
+Date_Job_Invoiced__c -&gt; invoice date (file cols 5/7)
+Total_Job_Amount__c -&gt; job amount (file col 12)
+Project_Name__c + Address__c -&gt; file col 13 (kept as separate fields)
+Vendor Name -&gt; file col 14 (account.name)
+Business_Flow_Type__c -&gt; actlink decode (file col 19)
+Line fields (Subie_Rate__c, Total_Actual_Amount__c, Item) -&gt; RCTI line detail</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Query validated in POC Test 3 (executed successfully incl. null-Vendor handling).
+Replaces the ODM_SS_STIFS flat-file extract — GL code, tax code and quantity move from hardcoded file values to SAP-side determination.
+Total_Job_Amount__c and Business_Flow_Type__c added beyond the Test 3 field list — confirm API names.
+Business flow fallback order (project -&gt; ticket -&gt; job) implemented in the iFlow mapping, not in SOQL.
+Negative amounts (credits) pass through as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>${lastSuccessfulPullTimestamp} = CPI variable holding the last successful pull timestamp. Pagination handled by the Salesforce adapter (validated in POC). Direct SiteTracker-to-CPI pattern — no Redshift.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A5:E5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4533,4 +4702,1125 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="130" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ODM (SiteTracker) Contract — Canonical Mapping and RCTI Extract Mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Adds the SiteTracker ODM contract to the INT-22 mapping pack. Two flows are covered:</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1. CREATE_SO — Service Order / WBS creation canonical, sourced from the ODM Project object (header.sourceMessageType is the constant 'CREATE_SO' for this table).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2. RCTI (supplier invoice) — the ODM_SS_STIFS_20260803_143008.csv extract is the current SiteTracker-to-IFS RCTI file; its columns are mapped on the 'ODM File Mapping' sheet and the replacement SAP CPI pull query is on 'ODM SOQL Queries' (validated in POC Test 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ODM_SS_STIFS_20260803_143008.csv — invoiced-job RCTI extract, 03/08/2026 run (107 lines). Row 1 of the file carries the source expressions (e.g. account.vendor_id__c, job.total_job_amount__c) rather than column names; the File Mapping sheet uses those expressions as the column identifiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Key observations from the data</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>- project_name formats seen: BRQ000000xxxxxx (BRQ works), NBN-0xxxxxxx (NBN remediation), DFN_xxxx_xxxx (DFN build) — project name + address are concatenated into one description field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>- map_to_actlink values seen: 1475PM, 1475RO, 1475SD — derived from business_flow_type__c (project, then ticket, then job — first value available). Candidate source for header.serviceHierarchy / workType decode; confirm code meanings with the FSM team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>- GL code 73020, GST10, quantity 1 and line_dissector 1 are hardcoded per line in the current extract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>- Negative amounts occur (e.g. J-051326, -126.67) — the RCTI canonical must support credit lines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>- CCR (Commercial Contract number) does not exist in SiteTracker yet — a field must be created to populate header.clientContractId (flagged GAP).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="75" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>FSM Field (SiteTracker ODM)</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Canonical Field (SAP Project)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Transformation</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Business Rule / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Constant 'CREATE_SO'</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>header.sourceMessageType</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Routing</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>This value must always equal CREATE_SO for this table — routes to the Service Order / WBS creation canonical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>projectName</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>header.fsmJobNumber</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Pass-through</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>SiteTracker project name (formats seen: BRQ000000xxxxxx, NBN-0xxxxxxx, DFN_xxxx).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>projectName</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>header.clientJobNumber</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Pass-through</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Same source as fsmJobNumber; populate when the client job reference equals the project name — confirm condition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>CCR (Commercial Contract number)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>header.clientContractId</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Pass-through</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Field to be CREATED in SiteTracker — no CCR field exists today. Drives Contract Mapping lookup. GAP until built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>workType (verify — may be costCode)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>header.serviceHierarchy</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Pass-through</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Verify whether the source is workType or costCode. The extract's map_to_actlink values (1475PM/1475RO/1475SD, derived from business_flow_type__c) are the candidate decode — confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>jobType</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>item.serviceHierarchy2</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Pass-through</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>header.state</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Pass-through</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Not a discrete field in the RCTI extract — currently only inside the concatenated address; needs a discrete source field on the Project object.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>header.customerRegion</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Pass-through</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Confirm source field on the Project object.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Col #</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Source Expression (file row 1)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Sample Value</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Maps To</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>1, 2, 3 ...</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>(technical — line counter)</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>NOT MAPPED</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>File line sequence only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>account.vendor_id__c</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>S047291 / V017247 / STOPSLO</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Supplier / vendor ID (RCTI canonical)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>MAPPED</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Matches sitetracker__Vendor__r.Vendor_ID__c validated in POC Test 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>job.name</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>J-021745</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Job reference (RCTI line key)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>MAPPED</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>SiteTracker Job ID — idempotency key for the invoice line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>job.name (duplicate)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>J-021745</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>(duplicate of col 3)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>NOT MAPPED</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Same value repeated for the legacy IFS layout; single field in the canonical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>job.date_job_invoiced__c</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>3/08/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Invoice date (RCTI canonical)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>MAPPED</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Matches Date_Job_Invoiced__c (Test 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>(unused)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>NOT MAPPED</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>job.date_job_invoiced__c (duplicate)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>3/08/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>(duplicate of col 5)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>NOT MAPPED</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Legacy layout duplicate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>hardcoded — line_dissector</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Line dissector</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Hardcoded 1 today; confirm whether multi-line dissection is required in the canonical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>hardcoded — gl_code</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>73020</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>GL account</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Hardcoded today; in SAP this should derive from the account-determination / Contract Mapping, not the file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>hardcoded — gst10</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>GST10</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Tax code</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Hardcoded GST10; confirm tax determination in S/4 replaces the hardcoding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>hardcoded — quantity</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Hardcoded 1 per job line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>job.total_job_amount__c</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>2255.24 / -126.67</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Line amount (RCTI canonical)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MAPPED</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Job-level invoiced amount. Negative values occur — credit lines must be supported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>project.project_name__c || ' ' || project.address__c</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>BRQ000000046205 25 Anzac Road Carina Heights QLD 4152</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>header.fsmJobNumber + description</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Concatenated in the extract. Canonical needs them SPLIT: project_name__c -&gt; header.fsmJobNumber / clientJobNumber; address (incl. state) as separate fields — pull separately in SOQL, do not parse the concat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>account.name</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>JAY BHAWANI CONSTRUCTION PTY LTD</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Supplier name</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>MAPPED</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Vendor account name; informational alongside vendor ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>(blank x4, cols 15-18)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>(unused)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>NOT MAPPED</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>map_to_actlink (business_flow_type__c: project, else ticket, else job)</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>1475PM / 1475RO / 1475SD</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>header.serviceHierarchy (workType decode)</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>First-available business flow type mapped to actlink code. Candidate source for serviceHierarchy — confirm code meanings (PM / RO / SD suffixes) with FSM team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>(blank x4, cols 20-23)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>(unused)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>NOT MAPPED</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>job.name</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>J-021745</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>(duplicate of col 3)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>NOT MAPPED</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Trailing legacy duplicate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>(no column)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>header.clientContractId (CCR)</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>CCR / Commercial Contract number absent from extract and from SiteTracker — field to be created.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>(no column)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>header.state</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>State only exists inside the concatenated address string — needs a discrete source field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>(no column)</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>header.customerRegion</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>No region column in the extract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>(no column)</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>item.serviceHierarchy2 (jobType)</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>No discrete jobType column in the extract — source from SiteTracker Job object in the SOQL pull.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
INT-22: consolidate ODM CREATE_SO and RCTI queries into main SOQL Queries sheet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NUogd2hZimCwR1pqCdqWGg
</commit_message>
<xml_diff>
--- a/INT-22_Contract_Reference_Mapping_20260805.xlsx
+++ b/INT-22_Contract_Reference_Mapping_20260805.xlsx
@@ -4483,7 +4483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4689,8 +4689,115 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="5" ht="300" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>ODM — CREATE_SO</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>ODM Service Order / WBS creation — pull new ODM projects</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       Project_Name__c,
+       Address__c,
+       Description__c,
+       Project_Start_A__c,
+       sitetracker__Project_Status__c,
+       Business_Flow_Type__c,
+       Work_Type__c,
+       Job_Type__c,
+       State__c,
+       Region__c,
+       CCR__c,
+       CreatedDate, LastModifiedDate
+FROM sitetracker__Project__c
+WHERE CreatedDate &gt;= ${lastSuccessfulPullTimestamp}</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Constant 'CREATE_SO' -&gt; header.sourceMessageType
+Project_Name__c -&gt; header.fsmJobNumber / header.clientJobNumber
+CCR__c -&gt; header.clientContractId
+Work_Type__c (or cost code) -&gt; header.serviceHierarchy
+Job_Type__c -&gt; item.serviceHierarchy2
+State__c -&gt; header.state
+Region__c -&gt; header.customerRegion</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Base project pull validated in POC (connectivity + delta query on sitetracker__Project__c).
+CCR__c does NOT exist yet — field to be created in SiteTracker (GAP).
+Work_Type__c / Job_Type__c / State__c / Region__c API names proposed from labels — confirm with Jackie; verify whether serviceHierarchy source is workType or costCode.
+Optionally filter on status (Active/Released) per requirements matrix row 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="300" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ODM — RCTI</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Supplier invoice — pull invoiced jobs + lines (replaces ODM_SS_STIFS file)</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       sitetracker__Job__c,
+       sitetracker__Job__r.Name,
+       sitetracker__Job__r.Project_Name__c,
+       sitetracker__Job__r.Date_Job_Invoiced__c,
+       sitetracker__Job__r.Total_Job_Amount__c,
+       sitetracker__Job__r.Business_Flow_Type__c,
+       sitetracker__Job__r.sitetracker__Vendor__r.Vendor_ID__c,
+       sitetracker__Job__r.sitetracker__Vendor__r.Name,
+       sitetracker__Job__r.Project__r.Project_Name__c,
+       sitetracker__Job__r.Project__r.Address__c,
+       Item_Name__r.Item_Id__c,
+       Item_Name__r.sitetracker__Primary_UoM__c,
+       Subie_Rate__c,
+       Total_Actual_Amount__c,
+       LastModifiedDate
+FROM sitetracker__Production_Plan_Line__c
+WHERE sitetracker__Job__r.sitetracker__Job_Status__c = 'Invoiced'
+  AND (LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp}
+       OR sitetracker__Job__r.LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp})</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Vendor_ID__c -&gt; supplier (file col 2, account.vendor_id__c)
+Job Name -&gt; invoice line key (file cols 3/4/24, job.name)
+Date_Job_Invoiced__c -&gt; invoice date (file cols 5/7)
+Total_Job_Amount__c -&gt; job amount (file col 12)
+Project_Name__c + Address__c -&gt; file col 13 (kept as separate fields)
+Vendor Name -&gt; file col 14 (account.name)
+Business_Flow_Type__c -&gt; actlink decode (file col 19)
+Line fields (Subie_Rate__c, Total_Actual_Amount__c, Item) -&gt; RCTI line detail</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Query validated in POC Test 3 (executed successfully incl. null-Vendor handling).
+Replaces the ODM_SS_STIFS flat-file extract — GL code, tax code and quantity move from hardcoded file values to SAP-side determination.
+Total_Job_Amount__c and Business_Flow_Type__c added beyond the Test 3 field list — confirm API names.
+Business flow fallback order (project -&gt; ticket -&gt; job) implemented in the iFlow mapping, not in SOQL.
+Negative amounts (credits) pass through as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>${lastSuccessfulPullTimestamp} = CPI variable holding the last successful pull timestamp (delta query). Pagination is handled by the Salesforce adapter (validated in POC). All queries target the direct SiteTracker-to-SAP-CPI pattern — no Redshift layer.</t>
         </is>
@@ -4698,7 +4805,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
INT-22: map ODM_SS_STIFS file data into ODM canonical mapping
Rebuild the ODM Canonical Mapping sheet canonical-first: each canonical
field now shows its ODM_SS_STIFS source column, real sample values from
the 03/08 run, and MAPPED/CONFIRM/GAP status.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NUogd2hZimCwR1pqCdqWGg
</commit_message>
<xml_diff>
--- a/INT-22_Contract_Reference_Mapping_20260805.xlsx
+++ b/INT-22_Contract_Reference_Mapping_20260805.xlsx
@@ -4934,15 +4934,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="75" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4973,6 +4976,21 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>ODM File Source (ODM_SS_STIFS_20260803)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Sample Value (03/08 file)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>Business Rule / Notes</t>
         </is>
       </c>
@@ -5005,6 +5023,21 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
+          <t>Not in file — constant set in the iFlow for this table.</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>CREATE_SO</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>MAPPED</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
           <t>This value must always equal CREATE_SO for this table — routes to the Service Order / WBS creation canonical.</t>
         </is>
       </c>
@@ -5037,199 +5070,318 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>SiteTracker project name (formats seen: BRQ000000xxxxxx, NBN-0xxxxxxx, DFN_xxxx).</t>
+          <t>Col 13 — project.project_name__c (first token of the concatenated 'project_name || address' field).</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>BRQ000000046205 / NBN-03674059 / DFN_3CWO_CW24_3CWO-65</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>MAPPED</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Three formats in the file: BRQ works, NBN- remediation, DFN_ build. Pull project_name__c as its own field in SOQL — do not parse the concatenated string.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>projectName</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>header.clientJobNumber</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Conditional</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Pass-through</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Same source as fsmJobNumber; populate when the client job reference equals the project name — confirm condition.</t>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Col 13 — same source as fsmJobNumber.</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>BRQ000000046205</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Populate when the client job reference equals the project name — confirm the condition per business flow.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>CCR (Commercial Contract number)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>header.clientContractId</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Pass-through</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Field to be CREATED in SiteTracker — no CCR field exists today. Drives Contract Mapping lookup. GAP until built.</t>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Not in file — no CCR column exists.</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Field to be CREATED in SiteTracker. Mandatory in the canonical, so this is a blocking gap; drives the Contract Mapping lookup.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>workType (verify — may be costCode)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>header.serviceHierarchy</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Conditional</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Pass-through</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Verify whether the source is workType or costCode. The extract's map_to_actlink values (1475PM/1475RO/1475SD, derived from business_flow_type__c) are the candidate decode — confirm.</t>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Col 19 — map_to_actlink, decoded from business_flow_type__c (project, else ticket, else job).</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>1475PM / 1475RO / 1475SD</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>CONFIRM</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Verify whether the canonical source is workType or costCode. The actlink codes are the closest field in the file — confirm the PM / RO / SD code meanings and whether they equal the workType decode.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>jobType</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>item.serviceHierarchy2</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Pass-through</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>No discrete column. Project-name prefix in col 13 indicates the job stream (BRQ / NBN- / DFN_).</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>BRQ-&gt;works, NBN-&gt;remediation, DFN-&gt;build (observed)</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Mandatory field with no discrete file source — source jobType from the SiteTracker Job object in the SOQL pull; the prefix pattern is an interim decode only, to be confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>header.state</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Pass-through</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Not a discrete field in the RCTI extract — currently only inside the concatenated address; needs a discrete source field on the Project object.</t>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Embedded in col 13 address text only (no discrete column).</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>QLD ('... Carina Heights QLD 4152') / VIC / NSW / ACT</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>States observed: QLD, VIC, NSW, ACT. Needs a discrete source field on the Project object — parsing the address string is not reliable (typos present in the data, e.g. 'Cabooulture').</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>header.customerRegion</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Conditional</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Pass-through</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Confirm source field on the Project object.</t>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Not in file.</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>No region column in the extract — confirm the source field on the Project object.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>File: ODM_SS_STIFS_20260803_143008.csv (107 invoiced-job lines, run 03/08/2026). Column numbers refer to the positional layout defined by the source expressions in file row 1. Fields not listed here (vendor ID/name, invoice date, job amount, GL/GST/quantity hardcodes) belong to the RCTI flow — see the ODM File Mapping sheet.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:I11"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
INT-22: final workbook — plain-English wording, validated runnable SOQL, gap highlighting
All five queries syntax-checked and made directly runnable (example
datetime literal replaces the CPI placeholder); READMEs and headers
rewritten in plain English; yellow = missing-field gap, orange = to
confirm, with legend on every query sheet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NUogd2hZimCwR1pqCdqWGg
</commit_message>
<xml_diff>
--- a/INT-22_Contract_Reference_Mapping_20260805.xlsx
+++ b/INT-22_Contract_Reference_Mapping_20260805.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -516,7 +516,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INT-22 WBSCreateUpdate — Contract Reference Mapping (SiteTracker / IFS extracts to SAP Canonical)</t>
+          <t>INT-22 — Contract Reference Mapping (SiteTracker to SAP)</t>
         </is>
       </c>
     </row>
@@ -526,14 +526,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>What this file is</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Revise the INT-22 contract reference mapping from multiple Site-tracker fields to single fields, and map the three contract data files to the SAP Project (WBS Create/Update) canonical model. Includes the SOQL pull queries for the SAP CPI Salesforce adapter to source the data directly from SiteTracker (per the agreed direct SiteTracker-to-CPI pattern — no Redshift layer).</t>
+          <t>For each contract, this file shows which field in the source data fills which field in SAP when a project and its work breakdown structure (WBS) are created or updated. It also contains the ready-to-run queries that SAP CI uses to pull the data straight from SiteTracker.</t>
         </is>
       </c>
     </row>
@@ -543,135 +543,149 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Source data files (05/08/2026)</t>
+          <t>Source data files (5 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>1. TLS_IFS_project_load_20260805.csv — Telstra contract project load (IFS)</t>
+          <t>1. TLS_IFS_project_load_20260805.csv — Telstra projects</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2. NBN_IFS_integration_20260805.csv — NBN Fixed Wireless project/activity extract (IFS)</t>
+          <t>2. NBN_IFS_integration_20260805.csv — NBN Fixed Wireless projects</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>3. Optus_1_meg2_projects_20260805.csv — Optus Meg2 projects/activity extract</t>
+          <t>3. Optus_1_meg2_projects_20260805.csv — Optus projects</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>4. ODM_SS_STIFS_20260803_143008.csv — ODM invoiced jobs (see the ODM sheets)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Sheets</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Canonical Mapping — INT-22 canonical model with per-contract SiteTracker source field (single field per contract).</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Sheets in this file</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TLS / NBN / Optus Field Mapping — every column in the contract data file mapped to the canonical field, with sample values, transformation and status.</t>
+          <t>Canonical Mapping — the full SAP field list, with the matching source field for each contract.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SOQL Queries — one delta pull query per contract for the SAP CPI Salesforce adapter (SiteTracker ODM).</t>
+          <t>TLS / NBN / Optus Field Mapping — every column in each data file, what it maps to, with real sample values.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>SOQL Queries — the five queries for SAP CI (Optus, Telstra, NBN, ODM project creation, ODM supplier invoices).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Legend</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ODM sheets — the same three views for the ODM contract.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Status = MAPPED: direct mapping confirmed from the data file.</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Status = CONFIRM (orange): mapping proposed — API/field name or business meaning to be confirmed (Jackie Pan / FSM team).</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Colour legend (used on every sheet)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Status = GAP (yellow): canonical field required but not present in the contract extract — must be sourced from SiteTracker or the Contract Mapping Table.</t>
+          <t>No colour — MAPPED: the source field is confirmed and ready to use.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Status = NOT MAPPED: file column not required by INT-22 (informational / contract master data).</t>
+          <t>ORANGE — CONFIRM: a mapping is proposed, but the field name or rule still needs to be confirmed.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>YELLOW — GAP: SAP needs this field but the source data does not have it yet. Someone must either create the field in SiteTracker or agree a different source.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Key assumptions</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>NOT MAPPED: the column is not needed for this integration.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>A1. header.clientContractId drives the Contract Mapping Table lookup (Profit Centre, Project Director, INT-21/INT-22 routing).</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>A2. header.isReleased and items[].isReleased are derived constants (auto-release in S/4), not sourced from the files.</t>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Working assumptions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>A3. Salesforce API names marked 'confirm' follow the labels validated in the Test 8/Test 9 POCs; remaining names to be confirmed against the SiteTracker org before build.</t>
+          <t>1. The contract ID on each message is used to look up the profit centre, project director and routing rules in the Contract Mapping Table.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>A4. Delta filter for all pull queries: LastModifiedDate &gt;= last successful pull timestamp; pagination handled by the Salesforce adapter (validated in POC).</t>
+          <t>2. Projects and WBS elements are released automatically in SAP — the release flags are set by the integration, not taken from the files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>3. Field names marked 'confirm' are proposed from screen labels and must be checked against the live SiteTracker system (Jackie Pan) before build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>4. Every query pulls only records created or changed since the last successful run.</t>
         </is>
       </c>
     </row>
@@ -689,7 +703,7 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="72" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
@@ -699,39 +713,39 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Contract / Flow</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>What it does</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>SOQL (SAP CPI Salesforce adapter)</t>
+          <t>Query to run in SAP CI (Salesforce adapter)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Field -&gt; Target</t>
+          <t>Which query field fills which SAP field</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Notes / To confirm</t>
+          <t>Things to check before build</t>
         </is>
       </c>
     </row>
     <row r="2" ht="300" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>CREATE_SO</t>
+          <t>ODM — project creation</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>ODM Service Order / WBS creation — pull new ODM projects</t>
+          <t>Pulls new ODM projects so SAP can create the service order and WBS (message type CREATE_SO).</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -750,38 +764,36 @@
        CCR__c,
        CreatedDate, LastModifiedDate
 FROM sitetracker__Project__c
-WHERE CreatedDate &gt;= ${lastSuccessfulPullTimestamp}</t>
+WHERE CreatedDate &gt;= 2026-08-01T00:00:00Z</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Constant 'CREATE_SO' -&gt; header.sourceMessageType
+          <t>Fixed value 'CREATE_SO' -&gt; header.sourceMessageType
 Project_Name__c -&gt; header.fsmJobNumber / header.clientJobNumber
 CCR__c -&gt; header.clientContractId
-Work_Type__c (or cost code) -&gt; header.serviceHierarchy
+Work_Type__c -&gt; header.serviceHierarchy
 Job_Type__c -&gt; item.serviceHierarchy2
 State__c -&gt; header.state
 Region__c -&gt; header.customerRegion</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Base project pull validated in POC (connectivity + delta query on sitetracker__Project__c).
-CCR__c does NOT exist yet — field to be created in SiteTracker (GAP).
-Work_Type__c / Job_Type__c / State__c / Region__c API names proposed from labels — confirm with Jackie; verify whether serviceHierarchy source is workType or costCode.
-Optionally filter on status (Active/Released) per requirements matrix row 1.</t>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>GAP: CCR__c does not exist in SiteTracker yet. SAP requires it, so the field must be created before this query can run as written.
+CHECK: Work_Type__c, Job_Type__c, State__c, Region__c field names; and whether serviceHierarchy should come from the work type or the cost code.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="300" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>RCTI</t>
+          <t>ODM — supplier invoices</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Supplier invoice — pull invoiced jobs + lines (replaces ODM_SS_STIFS file)</t>
+          <t>Pulls invoiced jobs and their lines. Replaces the current ODM_SS_STIFS flat file.</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -804,36 +816,36 @@
        LastModifiedDate
 FROM sitetracker__Production_Plan_Line__c
 WHERE sitetracker__Job__r.sitetracker__Job_Status__c = 'Invoiced'
-  AND (LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp}
-       OR sitetracker__Job__r.LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp})</t>
+  AND (LastModifiedDate &gt;= 2026-08-01T00:00:00Z
+       OR sitetracker__Job__r.LastModifiedDate &gt;= 2026-08-01T00:00:00Z)</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Vendor_ID__c -&gt; supplier (file col 2, account.vendor_id__c)
-Job Name -&gt; invoice line key (file cols 3/4/24, job.name)
-Date_Job_Invoiced__c -&gt; invoice date (file cols 5/7)
-Total_Job_Amount__c -&gt; job amount (file col 12)
-Project_Name__c + Address__c -&gt; file col 13 (kept as separate fields)
-Vendor Name -&gt; file col 14 (account.name)
-Business_Flow_Type__c -&gt; actlink decode (file col 19)
-Line fields (Subie_Rate__c, Total_Actual_Amount__c, Item) -&gt; RCTI line detail</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Query validated in POC Test 3 (executed successfully incl. null-Vendor handling).
-Replaces the ODM_SS_STIFS flat-file extract — GL code, tax code and quantity move from hardcoded file values to SAP-side determination.
-Total_Job_Amount__c and Business_Flow_Type__c added beyond the Test 3 field list — confirm API names.
-Business flow fallback order (project -&gt; ticket -&gt; job) implemented in the iFlow mapping, not in SOQL.
-Negative amounts (credits) pass through as-is.</t>
+          <t>Vendor_ID__c -&gt; supplier (file column 2)
+Job Name -&gt; invoice line key (file columns 3/4/24)
+Date_Job_Invoiced__c -&gt; invoice date (file columns 5/7)
+Total_Job_Amount__c -&gt; job amount (file column 12)
+Project_Name__c and Address__c -&gt; file column 13, kept as two separate fields
+Vendor Name -&gt; file column 14
+Business_Flow_Type__c -&gt; code decode (file column 19)
+Line fields (rate, amount, item) -&gt; invoice line detail</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Base query proven working in the Test 3 trial run, including jobs with no vendor.
+CHECK: Total_Job_Amount__c and Business_Flow_Type__c field names (added beyond the trial).
+The fallback order for the business flow code (project, then ticket, then job) is applied in the SAP CI mapping step, not in the query.
+The fixed account code, tax code and quantity in the old file are replaced by SAP's own determination.
+Negative amounts (credits) pass through unchanged.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>${lastSuccessfulPullTimestamp} = CPI variable holding the last successful pull timestamp. Pagination handled by the Salesforce adapter (validated in POC). Direct SiteTracker-to-CPI pattern — no Redshift.</t>
+          <t>The date 2026-08-01T00:00:00Z is an example only. In SAP CI, the integration flow replaces it on every run with the date and time of the last successful run, so only new or changed records are pulled. Large results are paged automatically by the Salesforce adapter. Colour legend: YELLOW = a needed field is missing at the source (gap). ORANGE = the field name or rule still needs to be confirmed before build.</t>
         </is>
       </c>
     </row>
@@ -871,12 +883,12 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>FSM Field</t>
+          <t>Source field (SiteTracker)</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Canonical Field (SAP Project)</t>
+          <t>SAP field</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -886,17 +898,17 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Required?</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>How the value is set</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Business Rule</t>
+          <t>Rule / meaning</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
@@ -2093,12 +2105,12 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Canonical Field (SAP Project)</t>
+          <t>SAP field</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>How the value is set</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -2923,12 +2935,12 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Canonical Field (SAP Project)</t>
+          <t>SAP field</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>How the value is set</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -3718,12 +3730,12 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Canonical Field (SAP Project)</t>
+          <t>SAP field</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>How the value is set</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -4486,7 +4498,7 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="72" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
@@ -4496,27 +4508,27 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Contract / Flow</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>What it does</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>SOQL (SAP CPI Salesforce adapter)</t>
+          <t>Query to run in SAP CI (Salesforce adapter)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Field -&gt; Canonical</t>
+          <t>Which query field fills which SAP field</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Notes / To confirm</t>
+          <t>Things to check before build</t>
         </is>
       </c>
     </row>
@@ -4528,7 +4540,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>INT-22 WBS Create/Update — pull new/changed Optus Megaladon projects</t>
+          <t>Pulls new and changed Optus projects for project / WBS creation.</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -4552,28 +4564,26 @@
 WHERE Client__c = 'Optus'
   AND Client_Status__c IN ('Current', 'Complete', 'On Hold')
   AND Program__c != '3G Partial Decom'
-  AND LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp}</t>
+  AND LastModifiedDate &gt;= 2026-08-01T00:00:00Z</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Name -&gt; canonicalProjectId derivation (P-xxxxxx)
+          <t>Name -&gt; project ID reference (P-xxxxxx)
 Site_ID__c -&gt; header.siteId
 sitetracker__Site_Name_Search__c -&gt; header.projectDescription
-WA_ID_Mirage__c -&gt; header.customerReference1 (WAID)
-Program__c -&gt; header.Program (Program Group)
+WA_ID_Mirage__c -&gt; header.customerReference1
+Program__c -&gt; header.Program
 State__c -&gt; header.State
-Client__c -&gt; Contract Mapping -&gt; header.clientContractId
-Phase_x flags -&gt; creation trigger conditions
-Design/SAED/Construction Code, CCR -&gt; item fields (add once API names confirmed)</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Base query validated in POC Test 8 (executed successfully via SAP CPI Salesforce adapter).
-State__c added beyond Test 8 list — confirm API name.
-Add WBS element fields (Design/SAED/Construction Code, CCR) once API names confirmed with Jackie.
-Delta filter + adapter pagination per POC.</t>
+Client__c -&gt; contract lookup -&gt; header.clientContractId
+Phase flags -&gt; creation trigger conditions</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Base query proven working in the Test 8 trial run.
+CHECK: State__c field name (it was not part of the trial).
+GAP: the WBS code fields (Design / SAED / Construction Code, CCR) are not in the query yet — add them once the field names are confirmed.</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4595,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>INT-22 WBS Create/Update — pull new/changed Telstra projects</t>
+          <t>Pulls new and changed Telstra projects for project / WBS creation.</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -4606,28 +4616,27 @@
 FROM sitetracker__Project__c
 WHERE Client__c = 'Telstra'
   AND Client_Status__c IN ('Current', 'Complete', 'On Hold')
-  AND LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp}</t>
+  AND LastModifiedDate &gt;= 2026-08-01T00:00:00Z</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Name -&gt; canonicalProjectId derivation (matches ST_Project_ID in file)
-Site_ID__c -&gt; header.siteId (Site_Id_A)
-sitetracker__Site_Name_Search__c -&gt; header.projectDescription (Site_Name_A)
+          <t>Name -&gt; project ID reference (matches ST_Project_ID in the file)
+Site_ID__c -&gt; header.siteId
+sitetracker__Site_Name_Search__c -&gt; header.projectDescription
 WA_ID_Mirage__c -&gt; header.customerReference1
-Program_ID__c -&gt; header.customerReference2 (Program ID)
+Program_ID__c -&gt; header.customerReference2
 Project_Office__c -&gt; header.State
-Work_Type__c -&gt; header.Program (Wo_Type)
+Work_Type__c -&gt; header.Program
 IFS_Detail_ID__c -&gt; items[].projectElement
 IFS_Build_ID__c -&gt; items[].projectElement3
-CP_No__c -&gt; items[].FSMJobID / clientContractId (Header_Contract_Ref)</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>API names for Program_ID__c, Project_Office__c, Work_Type__c, IFS_Detail_ID__c, IFS_Build_ID__c, CP_No__c are proposed from labels — confirm against the SiteTracker org (Jackie) before build.
-Confirm Client__c value for Telstra ('Telstra' vs 'TLS').
-IFS Detail/Build IDs fill the GAP rows in the TLS Field Mapping sheet.</t>
+CP_No__c -&gt; items[].FSMJobID</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>CHECK: six field names (Program_ID__c, Project_Office__c, Work_Type__c, IFS_Detail_ID__c, IFS_Build_ID__c, CP_No__c) are proposed from screen labels — confirm with Jackie before build.
+CHECK: whether the client value is stored as 'Telstra' or 'TLS'.</t>
         </is>
       </c>
     </row>
@@ -4639,7 +4648,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>INT-22 WBS Create/Update — pull new/changed NBN projects incl. ID66/ID164 milestone dates</t>
+          <t>Pulls new and changed NBN projects, including the ID66 start and ID164 end milestone dates.</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -4664,40 +4673,40 @@
 FROM sitetracker__Project__c
 WHERE Client__c = 'nbn'
   AND Client_Status__c IN ('Current', 'Complete', 'On Hold')
-  AND LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp}</t>
+  AND LastModifiedDate &gt;= 2026-08-01T00:00:00Z</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Name -&gt; canonicalProjectId derivation (matches project_id in file)
+          <t>Name -&gt; project ID reference (matches project_id in the file)
 Site_ID__c -&gt; header.siteId
 sitetracker__Site_Name_Search__c -&gt; header.projectDescription
-WA_ID_Mirage__c -&gt; header.customerReference1 (also basis for clientJobNumber)
+WA_ID_Mirage__c -&gt; header.customerReference1
 Job_Type__c -&gt; header.customerReference2
 State__c -&gt; header.State
 Program__c -&gt; header.Program
-Activity ID66 (Forecast/Actual) -&gt; items[].plannedStartDate
-Activity ID164 (Forecast/Actual) -&gt; items[].plannedEndDate</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Activity subquery pattern validated in POC Test 9 (sitetracker__Activity__c executed successfully).
-Confirm the parent-to-child relationship name (assumed sitetracker__Activities__r) and exact Activity Name values for ID66/ID164.
-Confirm Client__c value for NBN ('nbn' vs 'NBN').
-Job_Type__c API name proposed from label — confirm with Jackie.</t>
+ID66 activity dates -&gt; items[].plannedStartDate
+ID164 activity dates -&gt; items[].plannedEndDate</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Inner activity query proven working in the Test 9 trial run.
+CHECK: the child list name (assumed sitetracker__Activities__r) and the exact activity names for ID66/ID164.
+CHECK: whether the client value is stored as 'nbn' or 'NBN'.
+CHECK: Job_Type__c field name.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="300" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>ODM — CREATE_SO</t>
+          <t>ODM — project creation</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>ODM Service Order / WBS creation — pull new ODM projects</t>
+          <t>Pulls new ODM projects so SAP can create the service order and WBS (message type CREATE_SO).</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -4716,38 +4725,36 @@
        CCR__c,
        CreatedDate, LastModifiedDate
 FROM sitetracker__Project__c
-WHERE CreatedDate &gt;= ${lastSuccessfulPullTimestamp}</t>
+WHERE CreatedDate &gt;= 2026-08-01T00:00:00Z</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Constant 'CREATE_SO' -&gt; header.sourceMessageType
+          <t>Fixed value 'CREATE_SO' -&gt; header.sourceMessageType
 Project_Name__c -&gt; header.fsmJobNumber / header.clientJobNumber
 CCR__c -&gt; header.clientContractId
-Work_Type__c (or cost code) -&gt; header.serviceHierarchy
+Work_Type__c -&gt; header.serviceHierarchy
 Job_Type__c -&gt; item.serviceHierarchy2
 State__c -&gt; header.state
 Region__c -&gt; header.customerRegion</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Base project pull validated in POC (connectivity + delta query on sitetracker__Project__c).
-CCR__c does NOT exist yet — field to be created in SiteTracker (GAP).
-Work_Type__c / Job_Type__c / State__c / Region__c API names proposed from labels — confirm with Jackie; verify whether serviceHierarchy source is workType or costCode.
-Optionally filter on status (Active/Released) per requirements matrix row 1.</t>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>GAP: CCR__c does not exist in SiteTracker yet. SAP requires it, so the field must be created before this query can run as written.
+CHECK: Work_Type__c, Job_Type__c, State__c, Region__c field names; and whether serviceHierarchy should come from the work type or the cost code.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="300" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>ODM — RCTI</t>
+          <t>ODM — supplier invoices</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Supplier invoice — pull invoiced jobs + lines (replaces ODM_SS_STIFS file)</t>
+          <t>Pulls invoiced jobs and their lines. Replaces the current ODM_SS_STIFS flat file.</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -4770,36 +4777,36 @@
        LastModifiedDate
 FROM sitetracker__Production_Plan_Line__c
 WHERE sitetracker__Job__r.sitetracker__Job_Status__c = 'Invoiced'
-  AND (LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp}
-       OR sitetracker__Job__r.LastModifiedDate &gt;= ${lastSuccessfulPullTimestamp})</t>
+  AND (LastModifiedDate &gt;= 2026-08-01T00:00:00Z
+       OR sitetracker__Job__r.LastModifiedDate &gt;= 2026-08-01T00:00:00Z)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Vendor_ID__c -&gt; supplier (file col 2, account.vendor_id__c)
-Job Name -&gt; invoice line key (file cols 3/4/24, job.name)
-Date_Job_Invoiced__c -&gt; invoice date (file cols 5/7)
-Total_Job_Amount__c -&gt; job amount (file col 12)
-Project_Name__c + Address__c -&gt; file col 13 (kept as separate fields)
-Vendor Name -&gt; file col 14 (account.name)
-Business_Flow_Type__c -&gt; actlink decode (file col 19)
-Line fields (Subie_Rate__c, Total_Actual_Amount__c, Item) -&gt; RCTI line detail</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Query validated in POC Test 3 (executed successfully incl. null-Vendor handling).
-Replaces the ODM_SS_STIFS flat-file extract — GL code, tax code and quantity move from hardcoded file values to SAP-side determination.
-Total_Job_Amount__c and Business_Flow_Type__c added beyond the Test 3 field list — confirm API names.
-Business flow fallback order (project -&gt; ticket -&gt; job) implemented in the iFlow mapping, not in SOQL.
-Negative amounts (credits) pass through as-is.</t>
+          <t>Vendor_ID__c -&gt; supplier (file column 2)
+Job Name -&gt; invoice line key (file columns 3/4/24)
+Date_Job_Invoiced__c -&gt; invoice date (file columns 5/7)
+Total_Job_Amount__c -&gt; job amount (file column 12)
+Project_Name__c and Address__c -&gt; file column 13, kept as two separate fields
+Vendor Name -&gt; file column 14
+Business_Flow_Type__c -&gt; code decode (file column 19)
+Line fields (rate, amount, item) -&gt; invoice line detail</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Base query proven working in the Test 3 trial run, including jobs with no vendor.
+CHECK: Total_Job_Amount__c and Business_Flow_Type__c field names (added beyond the trial).
+The fallback order for the business flow code (project, then ticket, then job) is applied in the SAP CI mapping step, not in the query.
+The fixed account code, tax code and quantity in the old file are replaced by SAP's own determination.
+Negative amounts (credits) pass through unchanged.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>${lastSuccessfulPullTimestamp} = CPI variable holding the last successful pull timestamp (delta query). Pagination is handled by the Salesforce adapter (validated in POC). All queries target the direct SiteTracker-to-SAP-CPI pattern — no Redshift layer.</t>
+          <t>The date 2026-08-01T00:00:00Z is an example only. In SAP CI, the integration flow replaces it on every run with the date and time of the last successful run, so only new or changed records are pulled. Large results are paged automatically by the Salesforce adapter. Colour legend: YELLOW = a needed field is missing at the source (gap). ORANGE = the field name or rule still needs to be confirmed before build.</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4833,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ODM (SiteTracker) Contract — Canonical Mapping and RCTI Extract Mapping</t>
+          <t>ODM Contract — Mapping and Queries</t>
         </is>
       </c>
     </row>
@@ -4836,28 +4843,28 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>What the ODM sheets cover</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Adds the SiteTracker ODM contract to the INT-22 mapping pack. Two flows are covered:</t>
+          <t>Two flows for the ODM contract:</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. CREATE_SO — Service Order / WBS creation canonical, sourced from the ODM Project object (header.sourceMessageType is the constant 'CREATE_SO' for this table).</t>
+          <t>1. Project creation (CREATE_SO) — when a new project appears in SiteTracker, SAP creates the matching service order and work breakdown structure. The message type is always CREATE_SO for this table.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. RCTI (supplier invoice) — the ODM_SS_STIFS_20260803_143008.csv extract is the current SiteTracker-to-IFS RCTI file; its columns are mapped on the 'ODM File Mapping' sheet and the replacement SAP CPI pull query is on 'ODM SOQL Queries' (validated in POC Test 3).</t>
+          <t>2. Supplier invoices (RCTI) — today a flat file (ODM_SS_STIFS) is sent to the old system for invoiced jobs. The query on the ODM SOQL Queries sheet pulls the same data directly from SiteTracker instead.</t>
         </is>
       </c>
     </row>
@@ -4867,14 +4874,14 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Source file</t>
+          <t>About the data file</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ODM_SS_STIFS_20260803_143008.csv — invoiced-job RCTI extract, 03/08/2026 run (107 lines). Row 1 of the file carries the source expressions (e.g. account.vendor_id__c, job.total_job_amount__c) rather than column names; the File Mapping sheet uses those expressions as the column identifiers.</t>
+          <t>ODM_SS_STIFS_20260803_143008.csv — 107 invoiced-job lines from the 3 Aug 2026 run. The first row of the file holds the source formulas rather than column names, so the mapping sheets refer to columns by position.</t>
         </is>
       </c>
     </row>
@@ -4884,42 +4891,42 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Key observations from the data</t>
+          <t>What the data shows</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>- project_name formats seen: BRQ000000xxxxxx (BRQ works), NBN-0xxxxxxx (NBN remediation), DFN_xxxx_xxxx (DFN build) — project name + address are concatenated into one description field.</t>
+          <t>- Three project-name formats: BRQ… (works), NBN-… (remediation), DFN_… (build).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>- map_to_actlink values seen: 1475PM, 1475RO, 1475SD — derived from business_flow_type__c (project, then ticket, then job — first value available). Candidate source for header.serviceHierarchy / workType decode; confirm code meanings with the FSM team.</t>
+          <t>- The code in column 19 (1475PM / 1475RO / 1475SD) comes from the business flow type — first from the project, then the ticket, then the job, whichever has a value.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>- GL code 73020, GST10, quantity 1 and line_dissector 1 are hardcoded per line in the current extract.</t>
+          <t>- The account code (73020), tax code (GST10) and quantity (1) are fixed values written into every line of the current file. In SAP these will be determined by the system instead.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>- Negative amounts occur (e.g. J-051326, -126.67) — the RCTI canonical must support credit lines.</t>
+          <t>- Negative amounts appear (credits) — the new flow must accept them.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>- CCR (Commercial Contract number) does not exist in SiteTracker yet — a field must be created to populate header.clientContractId (flagged GAP).</t>
+          <t>- There is no commercial contract number (CCR) anywhere in SiteTracker yet. SAP requires it, so a new field must be created. This is the biggest gap.</t>
         </is>
       </c>
     </row>
@@ -4951,12 +4958,12 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>FSM Field (SiteTracker ODM)</t>
+          <t>Source field (SiteTracker ODM)</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Canonical Field (SAP Project)</t>
+          <t>SAP field</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -4966,12 +4973,12 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Required?</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Transformation</t>
+          <t>How the value is set</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -4991,7 +4998,7 @@
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>Business Rule / Notes</t>
+          <t>Rule / meaning</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5428,7 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Maps To</t>
+          <t>SAP field / use</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">

</xml_diff>

<commit_message>
INT-22: add DB validation queries sheet for all contracts
18 syntax-checked SQL reconciliation checks (Telstra, NBN, Optus, ODM
plus a cross-contract summary): record counts vs the SAP CI pull,
duplicate keys, missing required values, credit lines, and code lists.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NUogd2hZimCwR1pqCdqWGg
</commit_message>
<xml_diff>
--- a/INT-22_Contract_Reference_Mapping_20260805.xlsx
+++ b/INT-22_Contract_Reference_Mapping_20260805.xlsx
@@ -17,6 +17,7 @@
     <sheet name="ODM Canonical Mapping" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="ODM File Mapping" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="ODM SOQL Queries" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="DB Validation Queries" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,7 +65,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +85,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -140,6 +146,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -857,6 +866,523 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>What it checks</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>SQL query (run on the source database)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>What a good result looks like</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="70" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Telstra</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Row count in the load window</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) AS total_rows
+FROM tls_ifs_project_load
+WHERE load_date &gt;= DATE '2026-08-01';</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Must equal the number of records the SAP CI Telstra query returns for the same window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="70" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Telstra</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate project check</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>SELECT st_project_id, COUNT(*) AS copies
+FROM tls_ifs_project_load
+GROUP BY st_project_id
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>No rows. Any row listed is a duplicate project that would create the same SAP project twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="140" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Telstra</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Missing required values</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>SELECT
+  COUNT(*)                                AS total_rows,
+  COUNT(*) - COUNT(header_contract_ref)   AS missing_contract_ref,
+  COUNT(*) - COUNT(customer_project_id)   AS missing_job_number,
+  COUNT(*) - COUNT(site_id_a)             AS missing_site_id,
+  COUNT(*) - COUNT(site_name_a)           AS missing_site_name,
+  COUNT(*) - COUNT(program_id)            AS missing_program_id,
+  COUNT(*) - COUNT(project_director)      AS missing_project_director
+FROM tls_ifs_project_load;</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>All 'missing' columns should be 0. Any non-zero count means SAP will reject or misfile those records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Telstra</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Side-by-side compare with SAP</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>SELECT st_project_id, header_contract_ref, customer_project_id,
+       site_id_a, site_name_a, program_id, project_office,
+       wo_type, project_director
+FROM tls_ifs_project_load
+ORDER BY st_project_id;</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Line this up against the SAP CI query output (same fields, same order) — values must match row for row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>NBN</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Project count in the load window</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(DISTINCT project_id) AS projects
+FROM nbn_ifs_integration;</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Must equal the number of projects the SAP CI NBN query returns (the file has 2 activity rows per project).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NBN</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Design / construction row pairing</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>SELECT project_id,
+  SUM(CASE WHEN subcat = 'DN' THEN 1 ELSE 0 END) AS design_rows,
+  SUM(CASE WHEN subcat = 'CN' THEN 1 ELSE 0 END) AS construction_rows
+FROM nbn_ifs_integration
+GROUP BY project_id
+HAVING SUM(CASE WHEN subcat = 'DN' THEN 1 ELSE 0 END) &lt;&gt; 1
+    OR SUM(CASE WHEN subcat = 'CN' THEN 1 ELSE 0 END) &lt;&gt; 1;</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>No rows. Each project should have exactly one design (DN) row and one construction (CN) row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="126" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>NBN</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Missing required values</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>SELECT
+  COUNT(*)                              AS total_rows,
+  COUNT(*) - COUNT(customer)            AS missing_contract,
+  COUNT(*) - COUNT(customer_project)    AS missing_job_number,
+  COUNT(*) - COUNT(project_description) AS missing_site_name,
+  COUNT(*) - COUNT(state)               AS missing_state,
+  COUNT(*) - COUNT(program_id)          AS missing_program
+FROM nbn_ifs_integration;</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>All 'missing' columns should be 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>NBN</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>State code list (for the decode table)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>SELECT state, COUNT(*) AS rows_with_this_code
+FROM nbn_ifs_integration
+GROUP BY state
+ORDER BY state;</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Only expected codes (2, 3, 4 seen so far). A new code means the state decode table needs updating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Optus</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Project count in the load window</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(DISTINCT project_id) AS projects
+FROM optus_1_meg2_projects;</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Must equal the number of projects the SAP CI Optus query returns for the same window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Optus</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate project check</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>SELECT project_id, COUNT(*) AS copies
+FROM optus_1_meg2_projects
+GROUP BY project_id
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Rows here are expected only when a project has several activity lines — check they are activity rows, not true duplicates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="126" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Optus</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Missing required values</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>SELECT
+  COUNT(*)                              AS total_rows,
+  COUNT(*) - COUNT(customer_project)    AS missing_waid,
+  COUNT(*) - COUNT(site_id)             AS missing_site_id,
+  COUNT(*) - COUNT(project_description) AS missing_site_name,
+  COUNT(*) - COUNT(program_id)          AS missing_program_group,
+  COUNT(*) - COUNT(state)               AS missing_state
+FROM optus_1_meg2_projects;</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>All 'missing' columns should be 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Optus</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Excluded program check</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>SELECT program_id, program_description, COUNT(*) AS rows_in_program
+FROM optus_1_meg2_projects
+GROUP BY program_id, program_description
+ORDER BY rows_in_program DESC;</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Confirm no '3G Partial Decom' rows appear — the SAP CI query excludes that program, so the counts must be compared on the same basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="98" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>ODM</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Invoice totals by run date</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>SELECT date_job_invoiced,
+       COUNT(*)               AS invoice_lines,
+       SUM(total_job_amount)  AS total_amount
+FROM odm_ss_stifs
+GROUP BY date_job_invoiced
+ORDER BY date_job_invoiced;</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Line count and total amount must equal what the SAP CI supplier-invoice query returns for the same date. For the 3 Aug 2026 file: 107 lines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ODM</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate job check</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>SELECT job_name, COUNT(*) AS copies
+FROM odm_ss_stifs
+GROUP BY job_name
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>No rows. A duplicate job would create the same supplier invoice twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>ODM</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Missing supplier check</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>SELECT job_name, total_job_amount
+FROM odm_ss_stifs
+WHERE vendor_id IS NULL OR vendor_id = '';</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>No rows expected. Any row here is an invoice with no supplier — SAP cannot post it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ODM</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Credit lines (negative amounts)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>SELECT job_name, vendor_id, total_job_amount
+FROM odm_ss_stifs
+WHERE total_job_amount &lt; 0;</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Review each row — these are credits and must appear in SAP as credits, not be dropped. (One in the 3 Aug file: J-051326, -126.67.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ODM</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Business flow code list</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>SELECT map_to_actlink, COUNT(*) AS lines
+FROM odm_ss_stifs
+GROUP BY map_to_actlink
+ORDER BY map_to_actlink;</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Only expected codes (1475PM, 1475RO, 1475SD seen so far). A new code means the decode rule needs updating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="112" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>All contracts</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>One-line summary across sources</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>SELECT 'Telstra' AS contract, COUNT(*) AS rows_loaded FROM tls_ifs_project_load
+UNION ALL
+SELECT 'NBN', COUNT(DISTINCT project_id) FROM nbn_ifs_integration
+UNION ALL
+SELECT 'Optus', COUNT(DISTINCT project_id) FROM optus_1_meg2_projects
+UNION ALL
+SELECT 'ODM', COUNT(*) FROM odm_ss_stifs;</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>One row per contract. Compare each number with the record count from the matching SAP CI query run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>How to use: after each SAP CI run, run the matching checks on the source database and compare the numbers with what SAP received. Table and column names here follow the extract file headers (lower case, underscores) — swap them for the real table names in your database (for example the Redshift or staging schema) before running. The queries are standard SQL and run unchanged on Redshift, PostgreSQL and SQL Server (DATE '2026-08-01' becomes '2026-08-01' on SQL Server).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A21:D21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
INT-22: add local test database script + workbook sheet
Runnable SQL script (INT-22_local_test_db.sql) builds test tables for
all four contracts with real sample rows and runs the validation
checks; executed end-to-end locally with all checks returning expected
results. Same content added as a 'Local Test DB' workbook sheet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NUogd2hZimCwR1pqCdqWGg
</commit_message>
<xml_diff>
--- a/INT-22_Contract_Reference_Mapping_20260805.xlsx
+++ b/INT-22_Contract_Reference_Mapping_20260805.xlsx
@@ -18,6 +18,7 @@
     <sheet name="ODM File Mapping" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="ODM SOQL Queries" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="DB Validation Queries" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Local Test DB" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1383,6 +1384,257 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>SQL (copy into your local database)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>How to use</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>This sheet builds a small local test database for all four contracts so the validation queries can be tested before touching any real system. Each step creates one table matching the extract file layout and loads real sample rows from the Aug 2026 files. Run the steps in order, then run the checks in step 5 (same logic as the DB Validation Queries sheet). The full script is also saved in the repository as INT-22_local_test_db.sql — run it in one go with:  psql -d yourdb -f INT-22_local_test_db.sql   or   sqlite3 test.db &lt; INT-22_local_test_db.sql. The whole script has been executed end-to-end on a local database: all statements run and every check returns the expected result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="231" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>1. Telstra — create table + sample rows</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>DROP TABLE IF EXISTS tls_ifs_project_load;
+CREATE TABLE tls_ifs_project_load (
+  header_contract_ref   VARCHAR(20),
+  wo_type               VARCHAR(10),
+  customer_project_id_b VARCHAR(40),
+  site_id_b             VARCHAR(20),
+  site_name_a           VARCHAR(80),
+  customer_project_id   VARCHAR(40),
+  site_id_a             VARCHAR(20),
+  site_location         VARCHAR(10),
+  project_office        VARCHAR(20),
+  client                VARCHAR(10),
+  program_id            VARCHAR(10),
+  project_director      VARCHAR(50),
+  st_project_id         VARCHAR(20)
+);
+INSERT INTO tls_ifs_project_load VALUES
+('CP20004880','SMR','8350155257/1','034456','80 WOOD ROAD, TRUGANINA','8350155257-1','036677','VIC','National','TLS','TE6','BIBEKANANDA.NAG','P-036677'),
+('CP20004880','SAED','80005743/813','CTOH','CATOS HILL','VT23524','036293','TAS','VIC','TLS','TE0','BIBEKANANDA.NAG','P-036293');</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="286" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>2. NBN — create table + sample rows</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>DROP TABLE IF EXISTS nbn_ifs_integration;
+CREATE TABLE nbn_ifs_integration (
+  program_id            VARCHAR(10),
+  program_description   VARCHAR(60),
+  project_id            VARCHAR(20),
+  project_description   VARCHAR(80),
+  project_manager_engineer VARCHAR(50),
+  category_1            VARCHAR(10),
+  saed_scope            VARCHAR(20),
+  build_type            VARCHAR(20),
+  customer              VARCHAR(20),
+  customer_project      VARCHAR(40),
+  state                 VARCHAR(5),
+  activity              VARCHAR(10),
+  subcat                VARCHAR(5),
+  activity_id           VARCHAR(10),
+  activity_description  VARCHAR(60),
+  activity_category     VARCHAR(20)
+);
+INSERT INTO nbn_ifs_integration VALUES
+('17P012','NBN Fixed Wireless','P-011078','Wedderburn Reef',NULL,'DSC','FULL SAED','RF/MW OTHE','117NBN01','R302-3HRZ-3SOP-5106','3','712','DN','MS7040','Final Acceptance Complete','SAED'),
+('17P012','NBN Fixed Wireless','P-011078','Wedderburn Reef',NULL,'DSC','FULL SAED','RF/MW OTHE','117NBN01','R302-3HRZ-3SOP-5106','3','712','CN','MS7040','Final Acceptance Complete','Site Works'),
+('17P012','NBN Fixed Wireless','P-011083','Hayters Hill','Leo Orpilla','DSC',NULL,'RF/MW OTHE','117NBN01','R305-2GRZ-2BYB-5108','2','712','DN','MS7040','Final Acceptance Complete','SAED'),
+('17P012','NBN Fixed Wireless','P-011083','Hayters Hill','Leo Orpilla','DSC',NULL,'RF/MW OTHE','117NBN01','R305-2GRZ-2BYB-5108','2','712','CN','MS7040','Final Acceptance Complete','Site Works');</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="242" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>3. Optus — create table + sample rows</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>DROP TABLE IF EXISTS optus_1_meg2_projects;
+CREATE TABLE optus_1_meg2_projects (
+  program_id            VARCHAR(20),
+  program_description   VARCHAR(60),
+  project_id            VARCHAR(20),
+  project_description   VARCHAR(80),
+  project_manager_engineer VARCHAR(50),
+  category_1            VARCHAR(20),
+  category_2            VARCHAR(20),
+  customer              VARCHAR(20),
+  customer_project      VARCHAR(40),
+  state                 VARCHAR(5),
+  activity_description  VARCHAR(80),
+  site_id               VARCHAR(20),
+  saed_manager          VARCHAR(50)
+);
+INSERT INTO optus_1_meg2_projects VALUES
+('GRN-F-OO','Greenfield (OO)','P-018495','BULLABURRA','Muhammad Kashif','SAED','GRNFIELD_1','OPTUS','614022','1','phase_2_financial_milestones_complete','S0822','JAMES.BOUCHER'),
+('GRN-F-OO','Greenfield (OO)','P-015247','MARONG EAST','Muhammad Kashif','SAED','GRNFIELD_1','OPTUS','589330','1','phase_2_financial_milestones_complete','M4050','JAMES.BOUCHER'),
+('GRN-F-OO','Greenfield (OO)','P-018590','BELLMERE SOUTH','Brent Devin','SAED','GRNFIELD_1','OPTUS','615291','1','phase_2_financial_milestones_complete','B1958','JAMES.BOUCHER');</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="253" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>4. ODM — create table + sample rows</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>DROP TABLE IF EXISTS odm_ss_stifs;
+CREATE TABLE odm_ss_stifs (
+  line_no               INTEGER,
+  vendor_id             VARCHAR(20),
+  job_name              VARCHAR(20),
+  date_job_invoiced     VARCHAR(10),
+  line_dissector        INTEGER,
+  gl_code               VARCHAR(10),
+  tax_code              VARCHAR(10),
+  quantity              INTEGER,
+  total_job_amount      NUMERIC(12,2),
+  project_name_address  VARCHAR(200),
+  vendor_name           VARCHAR(120),
+  map_to_actlink        VARCHAR(10)
+);
+INSERT INTO odm_ss_stifs VALUES
+(1,'S047291','J-021745','2026-08-03',1,'73020','GST10',1,2255.24,'BRQ000000046205 25 Anzac Road Carina Heights QLD 4152','JAY BHAWANI CONSTRUCTION PTY LTD','1475PM'),
+(9,'S041047','J-039421','2026-08-03',1,'73020','GST10',1,6270.98,'NBN-03674059 50 HOWLEYS RD NOTTING HILL VIC 3168','AXIAL AIRCON PTY LTD','1475RO'),
+(17,'V017247','J-045498','2026-08-03',1,'73020','GST10',1,4708.98,'BRQ000000078821 63 Peel Street Wilton NSW 2571','Marsh Siban Pty Ltd','1475SD'),
+(16,'S043771','J-045424','2026-08-03',1,'73020','GST10',1,2100.98,'DFN_3CWO_CW24_3CWO-65 Near 292 Johnson St Abbotsford VIC 3067','THAT TELCO COMPANY PTY LTD','1475RO'),
+(107,'S033383','J-051326','2026-08-03',1,'73020','GST10',1,-126.67,'BRQ000000084272 174 Camden Road Douglas Park NSW 2569','J.P. COMMUNICATIONS','1475SD');</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="400" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>5. Validation checks (run after loading)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>-- Telstra: duplicate project check — expect no rows
+SELECT st_project_id, COUNT(*) AS copies
+FROM tls_ifs_project_load
+GROUP BY st_project_id
+HAVING COUNT(*) &gt; 1;
+-- Telstra: missing required values — expect all zeros
+SELECT
+  COUNT(*)                              AS total_rows,
+  COUNT(*) - COUNT(header_contract_ref) AS missing_contract_ref,
+  COUNT(*) - COUNT(customer_project_id) AS missing_job_number,
+  COUNT(*) - COUNT(site_id_a)           AS missing_site_id,
+  COUNT(*) - COUNT(site_name_a)         AS missing_site_name,
+  COUNT(*) - COUNT(program_id)          AS missing_program_id,
+  COUNT(*) - COUNT(project_director)    AS missing_project_director
+FROM tls_ifs_project_load;
+-- NBN: design / construction pairing — expect no rows
+SELECT project_id,
+  SUM(CASE WHEN subcat = 'DN' THEN 1 ELSE 0 END) AS design_rows,
+  SUM(CASE WHEN subcat = 'CN' THEN 1 ELSE 0 END) AS construction_rows
+FROM nbn_ifs_integration
+GROUP BY project_id
+HAVING SUM(CASE WHEN subcat = 'DN' THEN 1 ELSE 0 END) &lt;&gt; 1
+    OR SUM(CASE WHEN subcat = 'CN' THEN 1 ELSE 0 END) &lt;&gt; 1;
+-- NBN: state code list
+SELECT state, COUNT(*) AS rows_with_this_code
+FROM nbn_ifs_integration
+GROUP BY state
+ORDER BY state;
+-- Optus: missing required values — expect all zeros
+SELECT
+  COUNT(*)                              AS total_rows,
+  COUNT(*) - COUNT(customer_project)    AS missing_waid,
+  COUNT(*) - COUNT(site_id)             AS missing_site_id,
+  COUNT(*) - COUNT(project_description) AS missing_site_name,
+  COUNT(*) - COUNT(program_id)          AS missing_program_group,
+  COUNT(*) - COUNT(state)               AS missing_state
+FROM optus_1_meg2_projects;
+-- ODM: invoice totals by run date
+SELECT date_job_invoiced,
+       COUNT(*)              AS invoice_lines,
+       SUM(total_job_amount) AS total_amount
+FROM odm_ss_stifs
+GROUP BY date_job_invoiced
+ORDER BY date_job_invoiced;
+-- ODM: duplicate job check — expect no rows
+SELECT job_name, COUNT(*) AS copies
+FROM odm_ss_stifs
+GROUP BY job_name
+HAVING COUNT(*) &gt; 1;
+-- ODM: missing supplier — expect no rows
+SELECT job_name, total_job_amount
+FROM odm_ss_stifs
+WHERE vendor_id IS NULL OR vendor_id = '';
+-- ODM: credit lines — expect the known credit J-051326 only
+SELECT job_name, vendor_id, total_job_amount
+FROM odm_ss_stifs
+WHERE total_job_amount &lt; 0;
+-- ODM: business flow code list
+SELECT map_to_actlink, COUNT(*) AS lines
+FROM odm_ss_stifs
+GROUP BY map_to_actlink
+ORDER BY map_to_actlink;
+-- All contracts: one-line summary
+SELECT 'Telstra' AS contract, COUNT(*) AS rows_loaded FROM tls_ifs_project_load
+UNION ALL
+SELECT 'NBN', COUNT(DISTINCT project_id) FROM nbn_ifs_integration
+UNION ALL
+SELECT 'Optus', COUNT(DISTINCT project_id) FROM optus_1_meg2_projects
+UNION ALL
+SELECT 'ODM', COUNT(*) FROM odm_ss_stifs;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
INT-22: add SQL vs SOQL read-comparison sheet for all contracts
Read-only SQL for the SiteTracker reporting database paired with the
equivalent SOQL the SAP CPI adapter runs, per contract, with
comparison guidance. All SQL executed against a test schema.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NUogd2hZimCwR1pqCdqWGg
</commit_message>
<xml_diff>
--- a/INT-22_Contract_Reference_Mapping_20260805.xlsx
+++ b/INT-22_Contract_Reference_Mapping_20260805.xlsx
@@ -19,6 +19,7 @@
     <sheet name="ODM SOQL Queries" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="DB Validation Queries" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Local Test DB" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SQL vs SOQL (Read)" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1635,6 +1636,366 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Contract / Flow</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Read-only SQL — for Jackie to run on the SiteTracker reporting database</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Same query as SOQL — what the SAP CI Salesforce adapter runs</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>How to compare the two results</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="320" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Optus</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>SELECT id,
+       name,
+       site_id,
+       site_name_search,
+       wa_id_mirage,
+       program,
+       program_type,
+       project_engineer,
+       client,
+       client_status,
+       state,
+       phase_1_financial_milestones_complete,
+       phase_2_financial_milestones_complete,
+       phase_4_financial_milestones_complete,
+       saed_manager,
+       created_date,
+       last_modified_date
+FROM sitetracker_project
+WHERE client = 'Optus'
+  AND client_status IN ('Current', 'Complete', 'On Hold')
+  AND program &lt;&gt; '3G Partial Decom'
+  AND last_modified_date &gt;= '2026-08-01'
+ORDER BY name;</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       Site_ID__c,
+       sitetracker__Site_Name_Search__c,
+       WA_ID_Mirage__c,
+       Program__c,
+       Program_Type__c,
+       Project_Engineer__c,
+       Client__c,
+       Client_Status__c,
+       State__c,
+       Phase_1_Financial_Milestones_Complete__c,
+       Phase_2_Financial_Milestones_Complete__c,
+       Phase_4_Financial_Milestones_Complete__c,
+       SAED_Manager__c,
+       CreatedDate, LastModifiedDate
+FROM sitetracker__Project__c
+WHERE Client__c = 'Optus'
+  AND Client_Status__c IN ('Current', 'Complete', 'On Hold')
+  AND Program__c != '3G Partial Decom'
+  AND LastModifiedDate &gt;= 2026-08-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Row count and every field value must match. Both filter the same way: Optus client, allowed statuses, '3G Partial Decom' excluded, changed since 1 Aug 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="320" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Telstra</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>SELECT id,
+       name,
+       site_id,
+       site_name_search,
+       wa_id_mirage,
+       program_id,
+       project_office,
+       work_type,
+       ifs_detail_id,
+       ifs_build_id,
+       cp_no,
+       client,
+       client_status,
+       created_date,
+       last_modified_date
+FROM sitetracker_project
+WHERE client = 'Telstra'
+  AND client_status IN ('Current', 'Complete', 'On Hold')
+  AND last_modified_date &gt;= '2026-08-01'
+ORDER BY name;</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       Site_ID__c,
+       sitetracker__Site_Name_Search__c,
+       WA_ID_Mirage__c,
+       Program_ID__c,
+       Project_Office__c,
+       Work_Type__c,
+       IFS_Detail_ID__c,
+       IFS_Build_ID__c,
+       CP_No__c,
+       Client__c,
+       Client_Status__c,
+       CreatedDate, LastModifiedDate
+FROM sitetracker__Project__c
+WHERE Client__c = 'Telstra'
+  AND Client_Status__c IN ('Current', 'Complete', 'On Hold')
+  AND LastModifiedDate &gt;= 2026-08-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Row count and every field value must match. If the SQL side errors on a column name, that confirms the field name needs correcting on both sides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="320" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>NBN</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>SELECT p.id,
+       p.name,
+       p.site_id,
+       p.site_name_search,
+       p.wa_id_mirage,
+       p.job_type,
+       p.state,
+       p.program,
+       p.client,
+       p.client_status,
+       p.created_date,
+       p.last_modified_date,
+       a.name              AS activity_name,
+       a.forecast_actual   AS activity_forecast_date,
+       a.actual_date       AS activity_actual_date,
+       a.na                AS activity_not_applicable
+FROM sitetracker_project p
+LEFT JOIN sitetracker_activity a
+       ON a.project_id = p.id
+      AND a.name IN ('ID66 Site construction commencement (F)',
+                     'ID164 Operational Acceptance (F)')
+WHERE p.client = 'nbn'
+  AND p.client_status IN ('Current', 'Complete', 'On Hold')
+  AND p.last_modified_date &gt;= '2026-08-01'
+ORDER BY p.name, a.name;</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       Site_ID__c,
+       sitetracker__Site_Name_Search__c,
+       WA_ID_Mirage__c,
+       Job_Type__c,
+       State__c,
+       Program__c,
+       Client__c,
+       Client_Status__c,
+       CreatedDate, LastModifiedDate,
+       (SELECT Id, Name,
+               sitetracker__Forecast_Actual__c,
+               sitetracker__ActualDate__c,
+               sitetracker__NA__c
+        FROM sitetracker__Activities__r
+        WHERE Name IN ('ID66 Site construction commencement (F)',
+                       'ID164 Operational Acceptance (F)'))
+FROM sitetracker__Project__c
+WHERE Client__c = 'nbn'
+  AND Client_Status__c IN ('Current', 'Complete', 'On Hold')
+  AND LastModifiedDate &gt;= 2026-08-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Note the shape difference: the SQL returns one row per project per milestone activity (up to 2 rows per project); the SOQL returns one project record with the activities nested inside. Compare project counts and the ID66/ID164 dates per project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="320" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>ODM CREATE_SO</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>SELECT id,
+       name,
+       project_name,
+       address,
+       description,
+       project_start_a,
+       project_status,
+       business_flow_type,
+       work_type,
+       job_type,
+       state,
+       region,
+       ccr,
+       created_date,
+       last_modified_date
+FROM sitetracker_project
+WHERE created_date &gt;= '2026-08-01'
+ORDER BY name;</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       Project_Name__c,
+       Address__c,
+       Description__c,
+       Project_Start_A__c,
+       sitetracker__Project_Status__c,
+       Business_Flow_Type__c,
+       Work_Type__c,
+       Job_Type__c,
+       State__c,
+       Region__c,
+       CCR__c,
+       CreatedDate, LastModifiedDate
+FROM sitetracker__Project__c
+WHERE CreatedDate &gt;= 2026-08-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Row count and field values must match. The ccr column will error until the CCR field is created in SiteTracker — expected for now on both sides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="320" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>ODM RCTI</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>SELECT ppl.id,
+       ppl.name,
+       j.name                 AS job_name,
+       j.project_name,
+       j.date_job_invoiced,
+       j.total_job_amount,
+       j.business_flow_type,
+       v.vendor_id,
+       v.name                 AS vendor_name,
+       pr.project_name        AS parent_project_name,
+       pr.address             AS parent_project_address,
+       i.item_id,
+       i.primary_uom,
+       ppl.subie_rate,
+       ppl.total_actual_amount,
+       ppl.last_modified_date
+FROM sitetracker_production_plan_line ppl
+JOIN sitetracker_job j
+       ON j.id = ppl.job_id
+LEFT JOIN account v
+       ON v.id = j.vendor_id_ref
+LEFT JOIN sitetracker_project pr
+       ON pr.id = j.project_id
+LEFT JOIN sitetracker_item i
+       ON i.id = ppl.item_name_id
+WHERE j.job_status = 'Invoiced'
+  AND (ppl.last_modified_date &gt;= '2026-08-01'
+       OR j.last_modified_date &gt;= '2026-08-01')
+ORDER BY j.name;</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>SELECT Id, Name,
+       sitetracker__Job__c,
+       sitetracker__Job__r.Name,
+       sitetracker__Job__r.Project_Name__c,
+       sitetracker__Job__r.Date_Job_Invoiced__c,
+       sitetracker__Job__r.Total_Job_Amount__c,
+       sitetracker__Job__r.Business_Flow_Type__c,
+       sitetracker__Job__r.sitetracker__Vendor__r.Vendor_ID__c,
+       sitetracker__Job__r.sitetracker__Vendor__r.Name,
+       sitetracker__Job__r.Project__r.Project_Name__c,
+       sitetracker__Job__r.Project__r.Address__c,
+       Item_Name__r.Item_Id__c,
+       Item_Name__r.sitetracker__Primary_UoM__c,
+       Subie_Rate__c,
+       Total_Actual_Amount__c,
+       LastModifiedDate
+FROM sitetracker__Production_Plan_Line__c
+WHERE sitetracker__Job__r.sitetracker__Job_Status__c = 'Invoiced'
+  AND (LastModifiedDate &gt;= 2026-08-01T00:00:00Z
+       OR sitetracker__Job__r.LastModifiedDate &gt;= 2026-08-01T00:00:00Z)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Row count, job amounts and the sum of total_job_amount must match. Jobs with no supplier appear with empty vendor columns on both sides (left join = SOQL null relationship). Credits (negative amounts) must appear in both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Purpose: run the SQL (left) on the SiteTracker reporting database and the SOQL (right) through the SAP CI Salesforce adapter — the two result sets must match. Both queries are read-only; nothing is changed in any system. The SQL table and column names are the reporting-database versions of the Salesforce names (lower case, underscores, no __c) — adjust to the actual schema if it differs. The date '2026-08-01' is an example; use the same date on both sides when comparing. All five SQL queries have been executed against a test database to confirm they are valid; the five SOQL queries passed the same syntax checks earlier.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A8:D8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>